<commit_message>
backup before modify spatial dilation
</commit_message>
<xml_diff>
--- a/results/corr_groups_ALS.xlsx
+++ b/results/corr_groups_ALS.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[1, 12, 20, 28, 51, 57, 65, 104, 123, 126, 129, 131]</t>
+          <t>[0, 12, 21, 29, 50, 57, 65, 78, 102, 109, 129, 132, 135, 137]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[16, 17, 18, 19, 159, 160, 161, 210, 211, 212, 213, 269, 270, 271, 272, 273, 434, 435, 491, 492, 493, 494, 549, 550, 551, 907, 908, 909, 910, 911, 1092, 1093, 1094, 1095, 1113, 1114, 1115, 1167, 1168, 1169, 1170, 1183, 1184, 1185]</t>
+          <t>[16, 17, 18, 19, 159, 160, 161, 210, 211, 212, 213, 269, 270, 271, 272, 273, 434, 435, 492, 493, 494, 549, 550, 551, 658, 659, 847, 848, 907, 908, 909, 910, 911, 1092, 1093, 1094, 1095, 1113, 1114, 1115, 1167, 1168, 1169, 1170, 1183, 1184, 1185]</t>
         </is>
       </c>
     </row>
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[4, 29, 69, 85]</t>
+          <t>[3, 30, 69, 89]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -471,12 +471,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[5, 97]</t>
+          <t>[4, 90, 101]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[46, 842, 843]</t>
+          <t>[46, 784, 842, 843]</t>
         </is>
       </c>
     </row>
@@ -486,12 +486,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[6, 7, 8, 48, 49]</t>
+          <t>[5, 7, 8, 47, 48]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[77, 78, 79, 84, 85, 86, 87, 113, 114, 115, 419, 420, 421, 427, 428]</t>
+          <t>[77, 78, 79, 85, 86, 87, 113, 114, 115, 419, 420, 421, 427, 428]</t>
         </is>
       </c>
     </row>
@@ -501,12 +501,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[9, 18, 60, 63, 70, 73, 79, 89, 96, 101, 106, 115, 120]</t>
+          <t>[6, 80]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[144, 145, 146, 147, 201, 202, 203, 204, 509, 510, 511, 512, 519, 520, 601, 602, 603, 604, 641, 642, 643, 721, 722, 723, 801, 802, 803, 841, 842, 881, 882, 921, 922, 1025, 1026, 1027, 1028, 1029, 1076, 1077, 1078]</t>
+          <t>[84, 692, 693, 694]</t>
         </is>
       </c>
     </row>
@@ -516,12 +516,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[11, 35]</t>
+          <t>[9, 18, 60, 63, 70, 74, 82, 92, 100, 106, 111, 120, 125]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[150, 151, 348]</t>
+          <t>[144, 145, 146, 147, 201, 202, 203, 204, 509, 510, 511, 512, 519, 520, 601, 602, 603, 604, 641, 642, 643, 721, 722, 723, 801, 802, 803, 841, 842, 881, 882, 921, 922, 1025, 1026, 1027, 1028, 1029, 1076, 1077, 1078]</t>
         </is>
       </c>
     </row>
@@ -531,12 +531,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[13, 33, 36, 54, 91, 117, 125, 132]</t>
+          <t>[11, 35]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[177, 178, 179, 180, 181, 182, 322, 323, 324, 325, 349, 350, 467, 468, 811, 812, 813, 814, 1071, 1072, 1073, 1107, 1193, 1194, 1195]</t>
+          <t>[150, 151, 348]</t>
         </is>
       </c>
     </row>
@@ -546,12 +546,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[15, 39]</t>
+          <t>[13, 33, 36, 53, 94, 122, 131, 138]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[187, 375]</t>
+          <t>[177, 178, 179, 180, 181, 182, 322, 323, 324, 325, 349, 350, 467, 468, 811, 812, 813, 814, 1071, 1072, 1073, 1107, 1193, 1194, 1195]</t>
         </is>
       </c>
     </row>
@@ -561,12 +561,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[16, 26, 78]</t>
+          <t>[15, 40]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[190, 191, 243, 704]</t>
+          <t>[187, 375]</t>
         </is>
       </c>
     </row>
@@ -576,12 +576,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[23, 24, 44, 72]</t>
+          <t>[16, 27, 81]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[231, 232, 233, 234, 235, 236, 237, 238, 240, 241, 404, 405, 406, 407, 621, 622, 623, 624, 625]</t>
+          <t>[190, 191, 243, 704]</t>
         </is>
       </c>
     </row>
@@ -591,12 +591,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[25, 30, 38, 43, 68, 76, 99, 122]</t>
+          <t>[19, 108]</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[241, 242, 284, 285, 358, 359, 378, 379, 380, 573, 681, 682, 864, 865, 1090, 1091, 1092, 1093, 1094]</t>
+          <t>[204, 205, 896, 897, 898]</t>
         </is>
       </c>
     </row>
@@ -606,12 +606,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[34, 71, 105]</t>
+          <t>[20, 26, 31, 68, 79, 85, 110, 128]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[326, 327, 607, 608, 908, 909]</t>
+          <t>[206, 207, 208, 209, 241, 242, 284, 285, 573, 681, 682, 763, 764, 908, 909, 1091, 1092, 1093, 1094]</t>
         </is>
       </c>
     </row>
@@ -621,12 +621,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[40, 75, 84, 90, 93, 108, 124, 128]</t>
+          <t>[24, 25, 45, 73]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>[376, 655, 656, 780, 805, 825, 826, 944, 945, 1095, 1096, 1153, 1154]</t>
+          <t>[231, 232, 233, 234, 235, 236, 237, 238, 240, 241, 404, 405, 406, 407, 622, 623, 624, 625]</t>
         </is>
       </c>
     </row>
@@ -636,12 +636,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[52, 56]</t>
+          <t>[34, 46, 71, 104]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[437, 438, 439, 440, 441, 442, 443, 444, 445, 446, 447, 448, 449, 450, 451, 452, 453, 486, 487, 488]</t>
+          <t>[326, 327, 405, 607, 608, 864, 865]</t>
         </is>
       </c>
     </row>
@@ -651,12 +651,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[53, 81]</t>
+          <t>[41, 76, 88, 93, 97, 113, 130, 134]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[446, 727]</t>
+          <t>[376, 655, 656, 780, 805, 825, 826, 944, 945, 1095, 1096, 1153, 1154]</t>
         </is>
       </c>
     </row>
@@ -666,12 +666,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[62, 80, 111]</t>
+          <t>[51, 55]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[514, 723, 724, 725, 967]</t>
+          <t>[437, 438, 439, 440, 441, 442, 443, 444, 445, 446, 447, 448, 449, 450, 451, 452, 453, 486, 487, 488]</t>
         </is>
       </c>
     </row>
@@ -681,12 +681,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[74, 98]</t>
+          <t>[52, 84]</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[655, 656, 657, 658, 659, 847, 848, 849, 850]</t>
+          <t>[446, 727]</t>
         </is>
       </c>
     </row>
@@ -696,12 +696,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[86, 100]</t>
+          <t>[54, 123]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[784, 878]</t>
+          <t>[469, 1072]</t>
         </is>
       </c>
     </row>
@@ -711,12 +711,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[92, 94, 95]</t>
+          <t>[62, 83, 116]</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>[820, 821, 822, 823, 826, 827, 828, 829, 830, 838, 839]</t>
+          <t>[514, 723, 724, 725, 967]</t>
         </is>
       </c>
     </row>
@@ -726,12 +726,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[102, 121, 130]</t>
+          <t>[86, 114]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[885, 886, 887, 888, 1086, 1087, 1088, 1180, 1181]</t>
+          <t>[765, 766, 953, 954, 955]</t>
         </is>
       </c>
     </row>
@@ -741,12 +741,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>[103, 118]</t>
+          <t>[95, 98, 99]</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>[896, 897, 898, 1072]</t>
+          <t>[820, 821, 822, 823, 826, 827, 828, 829, 830, 838, 839]</t>
         </is>
       </c>
     </row>
@@ -756,12 +756,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>[107, 119]</t>
+          <t>[107, 126, 136]</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>[924, 1076]</t>
+          <t>[885, 886, 887, 888, 1086, 1087, 1088, 1180, 1181]</t>
         </is>
       </c>
     </row>
@@ -771,10 +771,25 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>[113, 116]</t>
+          <t>[112, 124]</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
+        <is>
+          <t>[924, 1076]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>[118, 121]</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>[1005, 1006, 1029]</t>
         </is>
@@ -791,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -817,7 +832,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[2, 17]</t>
+          <t>[1, 17]</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -832,12 +847,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[3, 42, 55, 58, 83, 88, 114]</t>
+          <t>[2, 58, 87, 91, 96, 119]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[27, 378, 469, 494, 771, 801, 1013]</t>
+          <t>[27, 494, 771, 801, 822, 1013]</t>
         </is>
       </c>
     </row>
@@ -847,12 +862,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[10, 14, 22, 109]</t>
+          <t>[10, 14, 23]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[146, 147, 179, 229, 953, 954, 955]</t>
+          <t>[146, 147, 179, 229]</t>
         </is>
       </c>
     </row>
@@ -862,12 +877,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[19, 82]</t>
+          <t>[22, 67]</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[204, 205, 206, 207, 208, 209, 763, 764, 765, 766]</t>
+          <t>[222, 556]</t>
         </is>
       </c>
     </row>
@@ -877,12 +892,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[21, 67]</t>
+          <t>[28, 44]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[222, 556]</t>
+          <t>[261, 379, 380]</t>
         </is>
       </c>
     </row>
@@ -892,12 +907,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[27, 45]</t>
+          <t>[32, 39, 43, 49, 61]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[261, 405]</t>
+          <t>[305, 358, 359, 378, 431, 511]</t>
         </is>
       </c>
     </row>
@@ -907,12 +922,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[32, 46, 50, 61]</t>
+          <t>[66, 127]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[305, 405, 431, 511]</t>
+          <t>[551, 552, 1090]</t>
         </is>
       </c>
     </row>
@@ -922,10 +937,25 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[110, 112]</t>
+          <t>[77, 103, 105]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>[657, 849, 850, 878]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>[115, 117]</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>[958, 959, 972, 973]</t>
         </is>
@@ -942,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -959,27 +989,27 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[284]</t>
+          <t>[356]</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[356, 357, 358]</t>
+          <t>[357]</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -989,11 +1019,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[405]</t>
+          <t>[491]</t>
         </is>
       </c>
     </row>
@@ -1019,39 +1049,29 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[551, 552]</t>
+          <t>[621]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[692, 693, 694]</t>
+          <t>[655, 656]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>87</v>
+        <v>133</v>
       </c>
       <c r="B10" t="inlineStr">
-        <is>
-          <t>[784]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>127</v>
-      </c>
-      <c r="B11" t="inlineStr">
         <is>
           <t>[1120, 1121, 1122]</t>
         </is>

</xml_diff>

<commit_message>
fix some bugs in 03
</commit_message>
<xml_diff>
--- a/results/corr_groups_ALS.xlsx
+++ b/results/corr_groups_ALS.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="39525" yWindow="3525" windowWidth="21600" windowHeight="13065" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="groups" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="centroid_groups" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="resting" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="zone_sizes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -52,7 +52,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -416,7 +416,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -792,7 +792,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -943,78 +943,706 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>joint_label</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>[356, 357]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>[377]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>[551, 552]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>70</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>[655, 656]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>74</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>[692, 693, 694]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>125</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>[1120, 1121, 1122]</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>joint_label</t>
+          <t>zone</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>frames</t>
+          <t>origin</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_members</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>pixel_area</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[356, 357]</t>
-        </is>
+          <t>group 0</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D2" t="n">
+        <v>130838</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[377]</t>
-        </is>
+          <t>group 1</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>111193</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[551, 552]</t>
-        </is>
+          <t>group 2</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>27925</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[655, 656]</t>
-        </is>
+          <t>group 3</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>46209</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[692, 693, 694]</t>
-        </is>
+          <t>group 4</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>157351</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[1120, 1121, 1122]</t>
-        </is>
+          <t>group 5</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>31269</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>group 6</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>119126</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>group 7</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5749</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>group 8</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>16412</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>group 9</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>20552</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>group 10</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>73880</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>group 11</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>164715</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>group 12</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="n">
+        <v>41809</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>group 13</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>17665</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>group 14</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>94087</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>group 15</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>6601</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>group 16</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>11048</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>group 17</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" t="n">
+        <v>10456</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>group 18</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>30598</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>group 19</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" t="n">
+        <v>141680</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>group 20</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>3</v>
+      </c>
+      <c r="D22" t="n">
+        <v>42771</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>group 21</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>8323</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>group 22</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>11516</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>centroid_group 0</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>35666</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>centroid_group 1</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="n">
+        <v>13922</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>centroid_group 2</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>23158</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>centroid_group 3</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>8592</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>centroid_group 4</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="n">
+        <v>30031</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>centroid_group 5</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>88509</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>centroid_group 6</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>centroid_group 7</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>35435</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>resting row 0</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>15261</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>resting row 1</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>4446</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>resting row 2</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>11134</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>resting row 3</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>124876</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>resting row 4</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>60341</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>resting row 5</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>71351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>